<commit_message>
Update pseudo-BoM, add AI model
Swapped bolts for a larger kit to include M2 for motor mount. Remove AS5047P encoder in favor for sensored BLDC motor. Add dupont / jumper wires. Add terminal breakout board for ESP32. Add Claude Sonnet 4.6 to AI attribution.
</commit_message>
<xml_diff>
--- a/doc/CAST_Proto1_Order.xlsx
+++ b/doc/CAST_Proto1_Order.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uconn-my.sharepoint.com/personal/anatol_gogoj_uconn_edu/Documents/Projects/CAST Spincoater/CAST/doc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{20B66776-69EC-4CE4-9550-B2350FD676F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="43" documentId="8_{20B66776-69EC-4CE4-9550-B2350FD676F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2CD81EBE-7F37-4C4B-8711-D31CA2D7900F}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="15634" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="5280" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CAST BoM" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="30">
   <si>
     <t>Designator</t>
   </si>
@@ -80,9 +80,6 @@
     <t>Flipsky ODESC V4.2 24V Single-Drive High-Current High-Precision Brushless Servo Motor Controller, FOC / BLDC, ODrivetool Compatible</t>
   </si>
   <si>
-    <t>AS5047P Magnetic Rotary Position Sensor / Encoder Breakout Board Module, SPI/ABI/UVW Outputs, 3.3V/5V Arduino Compatible (incl. magnet)</t>
-  </si>
-  <si>
     <t>SELOKY LM2596 DC-DC Buck Power Converter Module, Adjustable Voltage Regulator 4-40V to 1.25-37V (3PCS)</t>
   </si>
   <si>
@@ -101,9 +98,6 @@
     <t>Frame &amp; Mechanical</t>
   </si>
   <si>
-    <t>Kernmax 1120Pcs M3 Countersunk Screws Kit — M3 Flat Head Screws, Phillips Bolts Nuts Washers Set for 3D Printers</t>
-  </si>
-  <si>
     <t>Yaocom 300 Pcs M3 Threaded Inserts M3 x D5 x L4 Heat Set Inserts Brass for 3D Printing</t>
   </si>
   <si>
@@ -113,13 +107,22 @@
     <t>TOTAL</t>
   </si>
   <si>
-    <t>Rev 0  |  Feb 2026  |  All items purchased via Amazon.com</t>
-  </si>
-  <si>
     <t>CAST Spin Coater - Prototype Purchase Record</t>
   </si>
   <si>
     <t>Electronics / Motor Drive Subsystem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">900 Pcs Torx Countersunk Head Screws, M2 M2.5 M3 Bolts and Nuts Washers Set, Star Drive Flat Head Machine Screws, 304 Stainless Steel, Small Torx Bolts Fully Threaded with T6 T8 T10 Wrench </t>
+  </si>
+  <si>
+    <t>Rev 1  |  Mar 2026  |  All items purchased via Amazon.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3PCS ESP32 Breakout Board GPIO 1 into 2 Compatible with 30 Pins ESP32S ESP32 Development Board 2.4 GHz Dual Core WLAN WiFi + Bluetooth 2-in-1 Microcontroller ESP-WROOM-32 Chip for Arduino </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ELEGOO 120pcs Multicolored Dupont Wire 40pin Male to Female, 40pin Male to Male, 40pin Female to Female Breadboard Jumper Ribbon Cables Kit Compatible with Arduino Projects </t>
   </si>
 </sst>
 </file>
@@ -293,9 +296,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -303,53 +305,65 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -653,177 +667,177 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K25"/>
-  <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:G27"/>
+  <sheetFormatPr defaultColWidth="9.28515625" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12" style="2" customWidth="1"/>
-    <col min="2" max="2" width="62" style="2" customWidth="1"/>
-    <col min="3" max="3" width="10" style="2" customWidth="1"/>
-    <col min="4" max="4" width="8" style="2" customWidth="1"/>
-    <col min="5" max="6" width="13" style="2" customWidth="1"/>
-    <col min="7" max="7" width="12" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="9.23046875" style="2"/>
+    <col min="1" max="1" width="12" style="1" customWidth="1"/>
+    <col min="2" max="2" width="62" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10" style="1" customWidth="1"/>
+    <col min="4" max="4" width="8" style="1" customWidth="1"/>
+    <col min="5" max="6" width="13" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.28515625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:7" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-    </row>
-    <row r="4" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="7" t="s">
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+    </row>
+    <row r="4" spans="1:7" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="7" t="s">
+      <c r="B4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="8" t="s">
+    <row r="5" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-    </row>
-    <row r="6" spans="1:7" ht="42.45" x14ac:dyDescent="0.35">
-      <c r="A6" s="9"/>
-      <c r="B6" s="10" t="s">
+      <c r="B5" s="16"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="16"/>
+    </row>
+    <row r="6" spans="1:7" ht="42.75" x14ac:dyDescent="0.2">
+      <c r="A6" s="5"/>
+      <c r="B6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="9">
-        <v>1</v>
-      </c>
-      <c r="D6" s="9" t="s">
+      <c r="C6" s="5">
+        <v>1</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="7">
         <v>18.989999999999998</v>
       </c>
-      <c r="F6" s="11">
+      <c r="F6" s="7">
         <f>C6*E6</f>
         <v>18.989999999999998</v>
       </c>
-      <c r="G6" s="12" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="42.45" x14ac:dyDescent="0.35">
-      <c r="A7" s="13"/>
-      <c r="B7" s="14" t="s">
+      <c r="G6" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="42.75" x14ac:dyDescent="0.2">
+      <c r="A7" s="9"/>
+      <c r="B7" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="13">
-        <v>1</v>
-      </c>
-      <c r="D7" s="13" t="s">
+      <c r="C7" s="9">
+        <v>1</v>
+      </c>
+      <c r="D7" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="15">
+      <c r="E7" s="11">
         <v>20.99</v>
       </c>
-      <c r="F7" s="15">
+      <c r="F7" s="11">
         <f>C7*E7</f>
         <v>20.99</v>
       </c>
-      <c r="G7" s="16" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="8" t="s">
+      <c r="G7" s="12" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="57" x14ac:dyDescent="0.2">
+      <c r="A8" s="5"/>
+      <c r="B8" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-    </row>
-    <row r="10" spans="1:7" ht="28.3" x14ac:dyDescent="0.35">
-      <c r="A10" s="9"/>
-      <c r="B10" s="10" t="s">
+      <c r="C8" s="5">
+        <v>1</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" s="7">
+        <v>12.99</v>
+      </c>
+      <c r="F8" s="7">
+        <f>C8*E8</f>
+        <v>12.99</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
+    </row>
+    <row r="11" spans="1:7" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A11" s="5"/>
+      <c r="B11" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="9">
-        <v>1</v>
-      </c>
-      <c r="D10" s="9" t="s">
+      <c r="C11" s="5">
+        <v>1</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E10" s="11">
+      <c r="E11" s="7">
         <v>49.99</v>
       </c>
-      <c r="F10" s="11">
-        <f>C10*E10</f>
+      <c r="F11" s="7">
+        <f>C11*E11</f>
         <v>49.99</v>
       </c>
-      <c r="G10" s="12" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="42.45" x14ac:dyDescent="0.35">
-      <c r="A11" s="13"/>
-      <c r="B11" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="C11" s="13">
-        <v>1</v>
-      </c>
-      <c r="D11" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11" s="15">
-        <v>39.99</v>
-      </c>
-      <c r="F11" s="15">
-        <f>C11*E11</f>
-        <v>39.99</v>
-      </c>
-      <c r="G11" s="16" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="42.45" x14ac:dyDescent="0.35">
+      <c r="G11" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A12" s="9"/>
       <c r="B12" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C12" s="9">
         <v>1</v>
@@ -832,174 +846,174 @@
         <v>12</v>
       </c>
       <c r="E12" s="11">
-        <v>24.99</v>
+        <v>39.99</v>
       </c>
       <c r="F12" s="11">
         <f>C12*E12</f>
-        <v>24.99</v>
+        <v>39.99</v>
       </c>
       <c r="G12" s="12" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="28.3" x14ac:dyDescent="0.35">
-      <c r="A13" s="13"/>
-      <c r="B13" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" s="13">
-        <v>1</v>
-      </c>
-      <c r="D13" s="13" t="s">
+    <row r="13" spans="1:7" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A13" s="5"/>
+      <c r="B13" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="5">
+        <v>1</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E13" s="15">
+      <c r="E13" s="7">
         <v>9.99</v>
       </c>
-      <c r="F13" s="15">
+      <c r="F13" s="7">
         <f>C13*E13</f>
         <v>9.99</v>
       </c>
-      <c r="G13" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="8" t="s">
+      <c r="G13" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
+    </row>
+    <row r="16" spans="1:7" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A16" s="5"/>
+      <c r="B16" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-    </row>
-    <row r="16" spans="1:7" ht="28.3" x14ac:dyDescent="0.35">
-      <c r="A16" s="9"/>
-      <c r="B16" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="C16" s="9">
-        <v>1</v>
-      </c>
-      <c r="D16" s="9" t="s">
+      <c r="C16" s="5">
+        <v>1</v>
+      </c>
+      <c r="D16" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="7">
         <v>20.99</v>
       </c>
-      <c r="F16" s="11">
+      <c r="F16" s="7">
         <f>C16*E16</f>
         <v>20.99</v>
       </c>
-      <c r="G16" s="12" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="42.45" x14ac:dyDescent="0.35">
-      <c r="A17" s="13"/>
-      <c r="B17" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="C17" s="13">
-        <v>1</v>
-      </c>
-      <c r="D17" s="13" t="s">
+      <c r="G16" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="42.75" x14ac:dyDescent="0.2">
+      <c r="A17" s="9"/>
+      <c r="B17" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="9">
+        <v>1</v>
+      </c>
+      <c r="D17" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E17" s="15">
+      <c r="E17" s="11">
         <v>8.99</v>
       </c>
-      <c r="F17" s="15">
+      <c r="F17" s="11">
         <f>C17*E17</f>
         <v>8.99</v>
       </c>
-      <c r="G17" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="28.3" x14ac:dyDescent="0.35">
-      <c r="A18" s="9"/>
-      <c r="B18" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="C18" s="9">
-        <v>1</v>
-      </c>
-      <c r="D18" s="9" t="s">
+      <c r="G17" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="42.75" x14ac:dyDescent="0.2">
+      <c r="A18" s="5"/>
+      <c r="B18" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="5">
+        <v>1</v>
+      </c>
+      <c r="D18" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E18" s="11">
+      <c r="E18" s="7">
         <v>9.89</v>
       </c>
-      <c r="F18" s="11">
+      <c r="F18" s="7">
         <f>C18*E18</f>
         <v>9.89</v>
       </c>
-      <c r="G18" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-    </row>
-    <row r="21" spans="1:11" ht="28.3" x14ac:dyDescent="0.35">
-      <c r="A21" s="9"/>
-      <c r="B21" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="C21" s="9">
-        <v>1</v>
-      </c>
-      <c r="D21" s="9" t="s">
+      <c r="G18" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="57" x14ac:dyDescent="0.2">
+      <c r="A19" s="9"/>
+      <c r="B19" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C19" s="9">
+        <v>1</v>
+      </c>
+      <c r="D19" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E21" s="11">
-        <v>5.99</v>
-      </c>
-      <c r="F21" s="11">
-        <f>C21*E21</f>
-        <v>5.99</v>
-      </c>
-      <c r="G21" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" ht="28.3" x14ac:dyDescent="0.35">
-      <c r="A22" s="13"/>
-      <c r="B22" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="C22" s="13">
-        <v>1</v>
-      </c>
-      <c r="D22" s="13" t="s">
+      <c r="E19" s="11">
+        <v>6.98</v>
+      </c>
+      <c r="F19" s="11">
+        <f>C19*E19</f>
+        <v>6.98</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="16"/>
+      <c r="C21" s="16"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="16"/>
+      <c r="G21" s="16"/>
+    </row>
+    <row r="22" spans="1:7" ht="57" x14ac:dyDescent="0.2">
+      <c r="A22" s="5"/>
+      <c r="B22" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C22" s="5">
+        <v>1</v>
+      </c>
+      <c r="D22" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E22" s="15">
-        <v>9.99</v>
-      </c>
-      <c r="F22" s="15">
+      <c r="E22" s="7">
+        <v>9.59</v>
+      </c>
+      <c r="F22" s="7">
         <f>C22*E22</f>
-        <v>9.99</v>
+        <v>9.59</v>
       </c>
       <c r="G22" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="28.3" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A23" s="9"/>
       <c r="B23" s="10" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C23" s="9">
         <v>1</v>
@@ -1008,40 +1022,67 @@
         <v>9</v>
       </c>
       <c r="E23" s="11">
-        <v>4.95</v>
+        <v>9.99</v>
       </c>
       <c r="F23" s="11">
         <f>C23*E23</f>
+        <v>9.99</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A24" s="5"/>
+      <c r="B24" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C24" s="5">
+        <v>1</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E24" s="7">
         <v>4.95</v>
       </c>
-      <c r="G23" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="B25" s="18"/>
-      <c r="C25" s="18"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="18"/>
-      <c r="F25" s="19">
-        <f>SUM(F6:F7,F10:F13,F16:F18,F21:F23)</f>
-        <v>225.74000000000007</v>
-      </c>
-      <c r="G25" s="20"/>
-      <c r="H25" s="21"/>
-      <c r="I25" s="21"/>
-      <c r="J25" s="21"/>
-      <c r="K25" s="21"/>
+      <c r="F24" s="7">
+        <f>C24*E24</f>
+        <v>4.95</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A25" s="21"/>
+      <c r="B25" s="22"/>
+      <c r="C25" s="21"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="23"/>
+      <c r="F25" s="23"/>
+      <c r="G25" s="24"/>
+    </row>
+    <row r="27" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="B27" s="19"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="13">
+        <f>SUM(F6:F8,F11:F13,F16:F19,F22:F24)</f>
+        <v>224.32000000000005</v>
+      </c>
+      <c r="G27" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A9:G9"/>
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A21:G21"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A15:G15"/>
     <mergeCell ref="A5:G5"/>
@@ -1049,18 +1090,19 @@
   <hyperlinks>
     <hyperlink ref="G6" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="G7" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="G10" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="G11" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="G12" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="G13" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="G16" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="G17" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="G18" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="G21" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="G22" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="G23" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="G11" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="G12" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="G13" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="G16" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="G17" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="G18" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="G22" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="G23" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="G24" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="G8" r:id="rId12" xr:uid="{104D381D-73FF-49CF-8ED3-67E6AB96D881}"/>
+    <hyperlink ref="G19" r:id="rId13" xr:uid="{BAE5C983-2E25-4D02-83A8-77B68C999DA0}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId13"/>
+  <pageSetup orientation="portrait" r:id="rId14"/>
 </worksheet>
 </file>
</xml_diff>